<commit_message>
Fix end-to-end campaign selection, multi-campaign handling, and table pagination
</commit_message>
<xml_diff>
--- a/config/devices.xlsx
+++ b/config/devices.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,100 +436,15 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BR001</t>
+          <t>BR006</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Branch One</t>
+          <t>Bathinda</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
-        <is>
-          <t>B0077-chittorgarh-Midland Microfin Ltd,</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>BR002</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Jalandhar</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>B0001-Jalandhar-Midland Microfin Ltd, 170 Golden Avenue, kapila complex, First floor, Backside hotel kamal palace, garha road, Jalandhar Distt Jalandhar-144001 Punjab</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>BR003</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Ludhiana</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>B0003-LUDHIANA-Midland Microfin LTD, B-XX-2813 Gurdev nagar Pakhowal Road, Ranjit Tower,2nd building newer Park plaza Ludhiana Distt. Ludhiana-141001 State-Punjab</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>BR004</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Kapurthala</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>B0005-kapurthala-Midland Microfin Ltd, opp. Maan showroom, Taran taran road, Goindwal Sahib Distt. Taran Taran 143422 Punjab</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>BR005</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Hoshiarpur</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>B0006-Hoshiarpur-Midland Microfin Ltd, H.No.547/2, Street No.3, Near puri complex, Govt.College Road, Kamalpur, Hoshiarpur, Distt. HohiarpurPunjab- 146001</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>BR006</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Bathinda</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
         <is>
           <t>B0008-BATHINDA-Midland Microfin Ltd, 20554, Street No.23/A, Bansal Complex, Near Ghoda, Chowk, Ajit Road, Patti Mehna, Bathinda, Punjab.151001</t>
         </is>

</xml_diff>